<commit_message>
docs: budget 396 heures, materiel amorti et cout par mission
</commit_message>
<xml_diff>
--- a/docs/rendu/2026-09-23/CHIFFRAGE_ESTIME_REEL.xlsx
+++ b/docs/rendu/2026-09-23/CHIFFRAGE_ESTIME_REEL.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lots" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Méthode" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse déclarée" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lots'!$A$1:$L$19</definedName>
@@ -1427,4 +1428,130 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Déclaration équipe du 24/09/2026</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Personnes</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Heures/jour minimum</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Heures/soir approximatives</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Total reconstitué</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>B2*B3*(B4+B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Capacité initiale 5 personnes</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Écart heures</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>B6-B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ventilation par lot</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Non fournie : ne pas inventer</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Détail coût</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Voir COUTS_PRODUCTION.xlsx et 09_COUTS_PRODUCTION.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>